<commit_message>
Project completed - Clean up, service layer unit tests, some minor fixes and changes
</commit_message>
<xml_diff>
--- a/Flooring Mastery Peer Review 2.xlsx
+++ b/Flooring Mastery Peer Review 2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30105"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rjones\Documents\C382\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{87110D51-246C-4784-B63F-182989652B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A999A687-EFAD-47E4-8AD5-763E530D8CF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16485" yWindow="-15615" windowWidth="11655" windowHeight="13230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="53">
   <si>
     <t>Student</t>
   </si>
@@ -44,6 +44,12 @@
     <t>Reviewer</t>
   </si>
   <si>
+    <t>Zachary Therrian</t>
+  </si>
+  <si>
+    <t>Emmanuel Oviosa</t>
+  </si>
+  <si>
     <t>Code review form</t>
   </si>
   <si>
@@ -54,6 +60,9 @@
   </si>
   <si>
     <t>Does the code run?</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
   <si>
     <t>Run without errors (logical)</t>
@@ -629,13 +638,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="B2" s="8"/>
-      <c r="D2" s="9"/>
+    <row r="2" spans="1:4" ht="18.75">
+      <c r="B2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="3" spans="1:4" ht="26.1">
       <c r="A3" s="15" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="15"/>
@@ -649,10 +662,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="C5" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -660,17 +673,20 @@
         <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="B7" s="4" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="B8" s="4" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -678,6 +694,9 @@
         <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -686,17 +705,20 @@
         <v>3</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="B11" s="4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="B12" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -704,12 +726,15 @@
         <v>4</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>12</v>
+        <v>15</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="B14" s="5" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -717,226 +742,265 @@
         <v>5</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="B16" s="5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="B17" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="3">
         <v>6</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2">
+        <v>20</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="B19" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="B20" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" s="3">
         <v>7</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2">
+        <v>23</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="B22" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="B23" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
       <c r="A24" s="3">
         <v>8</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2">
+        <v>26</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
       <c r="B25" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
       <c r="B26" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" s="3">
         <v>9</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2">
+        <v>29</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
       <c r="B28" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
       <c r="A29" s="3">
         <v>10</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
+        <v>31</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
       <c r="A30" s="3">
         <v>11</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2">
+        <v>32</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
       <c r="A31" s="1"/>
       <c r="B31" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
       <c r="A32" s="3">
         <v>12</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2">
+        <v>34</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="B33" s="5" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="B34" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
       <c r="B35" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
       <c r="B36" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" s="3">
         <v>13</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2">
+        <v>39</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="B38" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
       <c r="B39" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
       <c r="A40" s="3">
         <v>14</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2">
+        <v>42</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="B41" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
       <c r="B42" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
       <c r="B43" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="B44" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
       <c r="A45" s="3">
         <v>15</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2">
+        <v>47</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
       <c r="A46" s="3">
         <v>16</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2">
+        <v>48</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
       <c r="B47" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
       <c r="A48" s="3">
         <v>17</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>47</v>
+        <v>50</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="49" spans="2:2">
       <c r="B49" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="50" spans="2:2">
       <c r="B50" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A3:D3"/>
   </mergeCells>
-  <conditionalFormatting sqref="C6:C50">
+  <conditionalFormatting sqref="C6:C35 C37:C50">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="No">
       <formula>NOT(ISERROR(SEARCH("No",C6)))</formula>
     </cfRule>

</xml_diff>